<commit_message>
change AMERICA NET to VERO
</commit_message>
<xml_diff>
--- a/arquivos/provedores_nuvem.xlsx
+++ b/arquivos/provedores_nuvem.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F257064\Documents\Codes\BLC TERCEIROS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F257064\Documents\Codes\BLC TERCEIROS\arquivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D63A7C86-54BD-4D75-93FC-B117BC2EAB38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04EB0DED-D197-4745-B824-9AA9FE29486B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
     <t>GIGA+</t>
   </si>
   <si>
-    <t>AMERICA NET</t>
+    <t>VERO</t>
   </si>
 </sst>
 </file>

</xml_diff>